<commit_message>
docs: translate to English and replace Graphify with Ripwire (task 36)
- Replace Graphify with Ripwire: delete graphify-out, commit
  ripwire-out/{graph.html,GRAPH_REPORT.md}, add npm run ripwire[:graph|:report],
  docs/ripwire.md, and a root AGENTS.md agent quick-start
- Rewrite docs/ARCHITECTURE_REVIEW.md around ripwire and update all references
- Translate API, database, raw-requirements, group-contract, meeting notes and
  remaining draft-task text to English; switch diacritic example to Polish
- Remove the course logbooks (docs/logbooks/) and fix dangling references
- Regenerate task-dependencies/task-gantt diagrams and the stakeholder report
- Correct stale demo captions (p2p/ledger) to the Solana topology
</commit_message>
<xml_diff>
--- a/docs/stakeholder-report.xlsx
+++ b/docs/stakeholder-report.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Changelog" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Tasks" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Questions" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Changelog" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Questions" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Tasks'!$A$1:$L$22</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Questions'!$A$1:$D$77</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Changelog'!$A$1:$E$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Tasks'!$A$1:$L$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Questions'!$A$1:$D$112</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -23,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -42,9 +43,6 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-    </font>
-    <font>
-      <i val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -72,12 +70,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -443,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -467,7 +464,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated 2026-09-03 08:13 UTC  |  matdevstamp/inl-3-awesome-journal</t>
+          <t>Generated 2026-10-11 17:09 UTC  |  matdevstamp/inl-3-awesome-journal</t>
         </is>
       </c>
     </row>
@@ -523,22 +520,22 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" t="n">
+        <v>19</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
         <v>4</v>
       </c>
-      <c r="D6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" t="n">
+      <c r="G6" t="n">
         <v>3</v>
-      </c>
-      <c r="F6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" t="n">
-        <v>20</v>
       </c>
     </row>
     <row r="7"/>
@@ -609,13 +606,13 @@
         <v>0</v>
       </c>
       <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
         <v>3</v>
       </c>
-      <c r="E10" t="n">
+      <c r="F10" t="n">
         <v>0</v>
-      </c>
-      <c r="F10" t="n">
-        <v>2</v>
       </c>
       <c r="G10" t="n">
         <v>0</v>
@@ -623,11 +620,7 @@
       <c r="H10" t="n">
         <v>2</v>
       </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>2026-09-04</t>
-        </is>
-      </c>
+      <c r="I10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -639,28 +632,24 @@
         <v>7</v>
       </c>
       <c r="C11" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="D11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E11" t="n">
+        <v>7</v>
+      </c>
+      <c r="F11" t="n">
         <v>0</v>
-      </c>
-      <c r="F11" t="n">
-        <v>1</v>
       </c>
       <c r="G11" t="n">
         <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>7</v>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>2026-09-05</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -672,13 +661,13 @@
         <v>6</v>
       </c>
       <c r="C12" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="D12" t="n">
         <v>0</v>
       </c>
       <c r="E12" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F12" t="n">
         <v>0</v>
@@ -687,13 +676,9 @@
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>6</v>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>2026-09-16</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -717,14 +702,14 @@
         <v>0</v>
       </c>
       <c r="G13" t="n">
+        <v>2</v>
+      </c>
+      <c r="H13" t="n">
         <v>0</v>
       </c>
-      <c r="H13" t="n">
-        <v>2</v>
-      </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -738,13 +723,13 @@
         <v>3</v>
       </c>
       <c r="C14" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D14" t="n">
         <v>0</v>
       </c>
       <c r="E14" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F14" t="n">
         <v>0</v>
@@ -753,111 +738,110 @@
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>3</v>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-    </row>
-    <row r="15"/>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+        <v>1</v>
+      </c>
+      <c r="I14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>16</v>
+      </c>
+      <c r="C15" t="n">
+        <v>16</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" t="n">
+        <v>2</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="16"/>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>Streams (ownership)</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>Stream</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>Tasks</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="C18" s="3" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr">
+      <c r="D18" s="3" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="E17" s="3" t="inlineStr">
+      <c r="E18" s="3" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
       </c>
-      <c r="F17" s="3" t="inlineStr">
+      <c r="F18" s="3" t="inlineStr">
         <is>
           <t>Blocked</t>
         </is>
       </c>
-      <c r="G17" s="3" t="inlineStr">
+      <c r="G18" s="3" t="inlineStr">
         <is>
           <t>Overdue</t>
         </is>
       </c>
-      <c r="H17" s="3" t="inlineStr">
+      <c r="H18" s="3" t="inlineStr">
         <is>
           <t>Next deadline</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>A-Identity</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>2</v>
-      </c>
-      <c r="C18" t="n">
-        <v>2</v>
-      </c>
-      <c r="D18" t="n">
-        <v>0</v>
-      </c>
-      <c r="E18" t="n">
-        <v>0</v>
-      </c>
-      <c r="F18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G18" t="n">
-        <v>0</v>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>2026-09-16</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>B-Patient</t>
+          <t>A-Identity</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D19" t="n">
         <v>0</v>
       </c>
       <c r="E19" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F19" t="n">
         <v>0</v>
@@ -865,29 +849,25 @@
       <c r="G19" t="n">
         <v>0</v>
       </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
+      <c r="H19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>C-Notes</t>
+          <t>B-Patient</t>
         </is>
       </c>
       <c r="B20" t="n">
         <v>1</v>
       </c>
       <c r="C20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D20" t="n">
         <v>0</v>
       </c>
       <c r="E20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F20" t="n">
         <v>0</v>
@@ -895,29 +875,25 @@
       <c r="G20" t="n">
         <v>0</v>
       </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
+      <c r="H20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>D-Audit</t>
+          <t>C-Notes</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C21" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D21" t="n">
         <v>0</v>
       </c>
       <c r="E21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F21" t="n">
         <v>0</v>
@@ -925,39 +901,61 @@
       <c r="G21" t="n">
         <v>0</v>
       </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>2026-09-16</t>
-        </is>
-      </c>
+      <c r="H21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>D-Audit</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="C22" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="D22" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F22" t="n">
         <v>0</v>
-      </c>
-      <c r="F22" t="n">
-        <v>3</v>
       </c>
       <c r="G22" t="n">
         <v>0</v>
       </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>2026-09-04</t>
+      <c r="H22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>31</v>
+      </c>
+      <c r="C23" t="n">
+        <v>18</v>
+      </c>
+      <c r="D23" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" t="n">
+        <v>13</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" t="n">
+        <v>4</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -972,14 +970,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -992,7 +990,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Compared against the snapshot of 2026-09-03 08:12 UTC</t>
+          <t>Compared against the snapshot of 2026-10-11 16:58 UTC</t>
         </is>
       </c>
     </row>
@@ -1025,13 +1023,145 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>No changes since the previous export.</t>
-        </is>
-      </c>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Questions</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>13 Patient View &amp; Search</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Question added</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>How to handle Polish characters in search? (ł, ż, ó)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Questions</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>13 Patient View &amp; Search</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Question removed</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>How to handle Swedish characters in search? (å, ä, ö)</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Questions</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>17 User Roles &amp; Access Control</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Question added</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>How to handle organization-based access for primary care centre? Answered: primary care centre is the login role</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Questions</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>17 User Roles &amp; Access Control</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Question removed</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>How to handle organization-based access for vårdcentral? Answered: vårdcentral is the login role</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Questions</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>36 Hackathon Documentation</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Question added</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Remove the course logbooks from the fork; keep `gruppkontrakt.md` and the meeting notes for honest provenance</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Questions</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>36 Hackathon Documentation</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Question removed</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Keep `gruppkontrakt.md` and the course logbooks in the fork, or remove them? Leaving them is honest; removing reduces noise</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:E10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1042,18 +1172,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L22"/>
+  <dimension ref="A1:L38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="39" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="37" customWidth="1" min="6" max="6"/>
+    <col width="47" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="48" customWidth="1" min="11" max="11"/>
     <col width="16" customWidth="1" min="12" max="12"/>
@@ -1140,7 +1270,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -1188,7 +1318,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -1235,22 +1365,22 @@
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Graphify Architecture Artifacts</t>
+          <t>Ripwire Architecture Artifacts</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Scaffold pair (Person 1 + Person 2)</t>
+          <t>Team (Gate 1 — Matias coordinates)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -1265,7 +1395,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>#30</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -1296,17 +1426,17 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>matdevstamp</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -1343,22 +1473,22 @@
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Vite + Tailwind CSS + shadcn/ui Setup</t>
+          <t>Next.js + Tailwind CSS + shadcn/ui Setup</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>matdevstamp</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -1372,7 +1502,11 @@
         </is>
       </c>
       <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>https://github.com/matdevstamp/inl-3-awesome-journal/issues/6</t>
+        </is>
+      </c>
       <c r="L6" t="n">
         <v>3</v>
       </c>
@@ -1391,22 +1525,22 @@
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Backend Project Setup</t>
+          <t>Backend Project Setup (Next.js Route Handlers &amp; Services)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>matdevstamp</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1416,11 +1550,15 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>#4, 05</t>
+          <t>#4, #6</t>
         </is>
       </c>
       <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>https://github.com/matdevstamp/inl-3-awesome-journal/issues/7</t>
+        </is>
+      </c>
       <c r="L7" t="n">
         <v>3</v>
       </c>
@@ -1444,17 +1582,17 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>matdevstamp</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1464,11 +1602,15 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>05, 06</t>
+          <t>#6, #7</t>
         </is>
       </c>
       <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>https://github.com/matdevstamp/inl-3-awesome-journal/issues/8</t>
+        </is>
+      </c>
       <c r="L8" t="n">
         <v>3</v>
       </c>
@@ -1492,12 +1634,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>matdevstamp</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1512,11 +1654,15 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>05, 07</t>
+          <t>#6, #8</t>
         </is>
       </c>
       <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>https://github.com/matdevstamp/inl-3-awesome-journal/issues/9</t>
+        </is>
+      </c>
       <c r="L9" t="n">
         <v>3</v>
       </c>
@@ -1540,17 +1686,17 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>matdevstamp</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1560,15 +1706,19 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>05, 06, 07, 08</t>
+          <t>#6, #7, #8, #9</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>10, 19</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr"/>
+          <t>#11, #29</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>https://github.com/matdevstamp/inl-3-awesome-journal/issues/10</t>
+        </is>
+      </c>
       <c r="L10" t="n">
         <v>4</v>
       </c>
@@ -1592,17 +1742,17 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>matdevstamp</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1612,15 +1762,19 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>05, 08, 07, 06</t>
+          <t>#6, #9, #8, #7</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>09</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr"/>
+          <t>#10</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>https://github.com/matdevstamp/inl-3-awesome-journal/issues/11</t>
+        </is>
+      </c>
       <c r="L11" t="n">
         <v>3</v>
       </c>
@@ -1648,17 +1802,17 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Kassim10</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1668,11 +1822,15 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>#4, 07, 06</t>
+          <t>#4, #8, #7</t>
         </is>
       </c>
       <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>https://github.com/matdevstamp/inl-3-awesome-journal/issues/13</t>
+        </is>
+      </c>
       <c r="L12" t="n">
         <v>4</v>
       </c>
@@ -1700,17 +1858,17 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>rcilomba</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1720,11 +1878,15 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>05, 07, 06</t>
+          <t>#6, #8, #7</t>
         </is>
       </c>
       <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>https://github.com/matdevstamp/inl-3-awesome-journal/issues/14</t>
+        </is>
+      </c>
       <c r="L13" t="n">
         <v>4</v>
       </c>
@@ -1752,17 +1914,17 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>rcilomba</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1772,15 +1934,19 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>#4, 11, 12</t>
+          <t>#4, #13, #14</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr"/>
+          <t>#16</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>https://github.com/matdevstamp/inl-3-awesome-journal/issues/15</t>
+        </is>
+      </c>
       <c r="L14" t="n">
         <v>4</v>
       </c>
@@ -1808,17 +1974,17 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Kassim10 (backend visibility) + rcilomba (UI)</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1828,15 +1994,19 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>#4, 11, 12</t>
+          <t>#4, #13, #14</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr"/>
+          <t>#15</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>https://github.com/matdevstamp/inl-3-awesome-journal/issues/16</t>
+        </is>
+      </c>
       <c r="L15" t="n">
         <v>4</v>
       </c>
@@ -1864,17 +2034,17 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>umoraghad0-del (huvudansvar, Stream D)</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1884,7 +2054,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>#4, 07, 06</t>
+          <t>#4, #8, #7</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -1892,7 +2062,11 @@
           <t>18</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr"/>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>https://github.com/matdevstamp/inl-3-awesome-journal/issues/17</t>
+        </is>
+      </c>
       <c r="L16" t="n">
         <v>4</v>
       </c>
@@ -1920,17 +2094,17 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>umoraghad0-del (pair-programmering)</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1940,11 +2114,15 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>15, 06</t>
+          <t>#17, #7</t>
         </is>
       </c>
       <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>https://github.com/matdevstamp/inl-3-awesome-journal/issues/18</t>
+        </is>
+      </c>
       <c r="L17" t="n">
         <v>4</v>
       </c>
@@ -1973,12 +2151,12 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>rcilomba</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1988,7 +2166,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>11, 12, 13, 14</t>
+          <t>#13, #14, #15, #16</t>
         </is>
       </c>
       <c r="J18" t="inlineStr"/>
@@ -2021,12 +2199,12 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>umoraghad0-del (pair-programmering)</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -2036,12 +2214,12 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>17, 14, 16, 12</t>
+          <t>#16, #18, #14, 17</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>#17</t>
         </is>
       </c>
       <c r="K19" t="inlineStr"/>
@@ -2068,17 +2246,17 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Team</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -2088,15 +2266,19 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>17, 15, 16, 18</t>
+          <t>#17, #18, 17, 18</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>09, 20</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr"/>
+          <t>#10, #30</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>https://github.com/matdevstamp/inl-3-awesome-journal/issues/29</t>
+        </is>
+      </c>
       <c r="L20" t="n">
         <v>4</v>
       </c>
@@ -2120,12 +2302,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Kassim10</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -2145,10 +2327,14 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>#3, 19</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr"/>
+          <t>#3, #29</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>https://github.com/matdevstamp/inl-3-awesome-journal/issues/30</t>
+        </is>
+      </c>
       <c r="L21" t="n">
         <v>4</v>
       </c>
@@ -2172,12 +2358,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Team</t>
+          <t>Kassim10</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -2192,17 +2378,845 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>19, 09, 20</t>
+          <t>#29, #10, #30</t>
         </is>
       </c>
       <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>https://github.com/matdevstamp/inl-3-awesome-journal/issues/31</t>
+        </is>
+      </c>
       <c r="L22" t="n">
         <v>4</v>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Solana Repo Split and Toolchain</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>matdevstamp</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>5h</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Freeze the Interface Contract</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>matdevstamp</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>3h</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>24, 25</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Solana Program Scaffold</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>matdevstamp</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>4h</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Pure Hash Chain Module</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>matdevstamp</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>5h</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Durable Outbox and Solana Flusher</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>matdevstamp</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>9h</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Build the Anchor Program</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>matdevstamp</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>5h</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>24, 25</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>28, 29</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Devnet Deploy</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>matdevstamp</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>2h</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Solana Program Tests</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>matdevstamp</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>7h</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>27, 28</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr"/>
+      <c r="L30" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Solana Client and Environment</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>matdevstamp</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>5h</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>27, 28</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Remove the Homemade Blockchain</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>matdevstamp</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>6h</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Wire Flusher to the Solana Program</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>matdevstamp</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>5h</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>31, 30</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr"/>
+      <c r="L33" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Patient Wallet Integration</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>matdevstamp</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>6h</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr"/>
+      <c r="L34" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr"/>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Solana Verification UI</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>matdevstamp</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>6h</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr"/>
+      <c r="L35" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>E2E and Submission Disclosure</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>matdevstamp</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>4h</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>29, 32</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>36, 37</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr"/>
+      <c r="L36" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr"/>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Hackathon Documentation</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>matdevstamp</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>5h</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>35, 37</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr"/>
+      <c r="L37" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr"/>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Hackathon Submission and Decks</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>matdevstamp</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>13h</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>35, 36</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr"/>
+      <c r="L38" t="n">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L22"/>
+  <autoFilter ref="A1:L38"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2213,11 +3227,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D77"/>
+  <dimension ref="A1:D112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="2" max="2"/>
     <col width="48" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
   </cols>
@@ -2257,12 +3271,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Which frontend framework will we use? (React, Vue, Svelte?)</t>
+          <t>Frontend: React inside Next.js (fullstack) — decided at kickoff</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2279,12 +3293,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Which authentication method? (JWT, sessions, passwordless?)</t>
+          <t>Auth: JWT in an httpOnly cookie — decided at kickoff</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2301,12 +3315,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>How will we handle the blockchain implementation?</t>
+          <t>Blockchain: simple custom chain (stream D split TBD) — decided at kickoff</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2323,12 +3337,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>What database will we use? (PostgreSQL, MySQL, SQLite?)</t>
+          <t>Database: PostgreSQL (dev + prod) — decided at kickoff</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2345,12 +3359,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Which database do we choose? (SQLite, PostgreSQL, or both?)</t>
+          <t>Which database do we choose? → **PostgreSQL** (dev and prod)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2372,7 +3386,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2394,7 +3408,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2416,7 +3430,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2428,17 +3442,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>03 Graphify Architecture Artifacts</t>
+          <t>03 Ripwire Architecture Artifacts</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Which graphify version and command will be documented in the README?</t>
+          <t>Which ripwire version and command will be documented in the README? Answer: `npm run ripwire` (ripwire 0.5.0), see `docs/ripwire.md`.</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2455,12 +3469,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>PostgreSQL vs SQLite? (see task 02-database-choice-discussion.md)</t>
+          <t>PostgreSQL vs SQLite? → **PostgreSQL** (see task 02-database-choice-discussion.md)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2477,12 +3491,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Should we use Prisma as the single source of truth?</t>
+          <t>Prisma as single source of truth? → yes; DBML dropped</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2504,7 +3518,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2526,7 +3540,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2538,7 +3552,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>05 Vite + Tailwind CSS + shadcn/ui Setup</t>
+          <t>05 Next.js + Tailwind CSS + shadcn/ui Setup</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2548,7 +3562,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2560,7 +3574,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>05 Vite + Tailwind CSS + shadcn/ui Setup</t>
+          <t>05 Next.js + Tailwind CSS + shadcn/ui Setup</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2570,7 +3584,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2582,7 +3596,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>05 Vite + Tailwind CSS + shadcn/ui Setup</t>
+          <t>05 Next.js + Tailwind CSS + shadcn/ui Setup</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2592,7 +3606,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2604,17 +3618,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>06 Backend Project Setup</t>
+          <t>06 Backend Project Setup (Next.js Route Handlers &amp; Services)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>PostgreSQL vs SQLite for development?</t>
+          <t>PostgreSQL vs SQLite for development? → PostgreSQL (task 02 decision)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2626,17 +3640,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>06 Backend Project Setup</t>
+          <t>06 Backend Project Setup (Next.js Route Handlers &amp; Services)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Which ORM to use? (Prisma recommended)</t>
+          <t>Which ORM to use? → Prisma</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2648,7 +3662,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>06 Backend Project Setup</t>
+          <t>06 Backend Project Setup (Next.js Route Handlers &amp; Services)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2658,7 +3672,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2680,7 +3694,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2702,7 +3716,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2724,7 +3738,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2746,7 +3760,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2768,7 +3782,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2790,7 +3804,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2812,7 +3826,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2834,7 +3848,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2856,7 +3870,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2878,7 +3892,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2900,7 +3914,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2917,12 +3931,12 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Which hosting platform for deployment?</t>
+          <t>Should we run E2E tests in CI from the start or only near Gate 4?</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2939,12 +3953,12 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Should we run E2E tests in CI?</t>
+          <t>Can the ruleset enforce the docs-direct carve-out per path?</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2961,12 +3975,12 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>JWT vs session-based auth? (JWT recommended for simplicity)</t>
+          <t>JWT vs session-based auth? → JWT in httpOnly cookie (kickoff)</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3027,12 +4041,12 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Should we use an API framework like Fastify instead of Express?</t>
+          <t>Express vs another framework? → no Express; Next.js route handlers (kickoff)</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3049,12 +4063,12 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>React vs Vue vs Svelte? (React recommended)</t>
+          <t>React vs Vue vs Svelte? → React in Next.js (kickoff)</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3071,12 +4085,12 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Which CSS framework? (Tailwind recommended)</t>
+          <t>Which CSS framework? → Tailwind + shadcn/ui (kickoff)</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3093,12 +4107,12 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>State management approach? (Context API vs Redux)</t>
+          <t>State management approach? → custom useSyncExternalStore session store; TanStack Query not adopted (PR #24)</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3115,12 +4129,12 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Should we use a component library? (Material UI, Ant Design?)</t>
+          <t>Component library? → shadcn/ui (kickoff)</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3137,7 +4151,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>How to handle Swedish characters in search? (å, ä, ö)</t>
+          <t>How to handle Polish characters in search? (ł, ż, ó)</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -3489,12 +4503,12 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>How to handle organization-based access for vårdcentral?</t>
+          <t>How to handle organization-based access for primary care centre? Answered: primary care centre is the login role</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3577,7 +4591,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Should we use Redis adapter for scaling?</t>
+          <t>Should we use Redis adapter for scaling? (open — single-pair demo works without it)</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -3599,12 +4613,12 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>How to handle socket authentication?</t>
+          <t>How to handle socket authentication? (JWT session cookie verified at handshake + peer shared secret for P2P calls)</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3621,12 +4635,12 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>What's the reconnection strategy?</t>
+          <t>What's the reconnection strategy? (socket.io-client auto-reconnect, 5 attempts, client-side note dedup on resync)</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3643,7 +4657,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Should we implement message acknowledgments?</t>
+          <t>Should we implement message acknowledgments? (open — current flow relies on client-side dedup instead)</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -3665,12 +4679,12 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Which testing framework to use? (Jest recommended for Node.js)</t>
+          <t>Which testing framework to use? → Vitest (unit/integration) + Playwright (E2E), matching task 09.</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3687,12 +4701,12 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>How to set up test database?</t>
+          <t>How to set up test database? → Docker Postgres via `e2e/global-setup.ts`, migrated and seeded per run.</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3709,12 +4723,12 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Should we implement E2E tests with Cypress?</t>
+          <t>Should we implement E2E tests with Cypress? → No, Playwright was already chosen in task 09.</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3731,12 +4745,12 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>How to handle socket.io testing?</t>
+          <t>How to handle socket.io testing? → Two `next start` instances (3001/3002) with real Socket.io ports; cross-server delivery is asserted over a WebSocket client.</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3775,12 +4789,12 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>How detailed should API documentation be?</t>
+          <t>How detailed should API documentation be? → route-handler table in README</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3797,12 +4811,12 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Should we use a documentation generator (e.g., Swagger)?</t>
+          <t>Should we use a documentation generator? → no (shared types; kickoff)</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3819,12 +4833,12 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>How to format meeting notes consistently?</t>
+          <t>How to format meeting notes consistently? → `YYYY-MM-DD-&lt;meeting-type&gt;.md`; use the structure in [`docs/MEETING_TEMPLATE.md`](../MEETING_TEMPLATE.md) and keep raw transcripts in `docs/meetings/archive/`.</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3916,8 +4930,778 @@
         </is>
       </c>
     </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>22 Solana Repo Split and Toolchain</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Does `anchor build` require platform tools (`cargo install --locked --git https://github.com/anza-xyz/platform-tools`)?</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>22 Solana Repo Split and Toolchain</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Which devnet RPC provider for E2E? The public endpoint rate-limits under parallel tests</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>23 Freeze the Interface Contract</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Does Anchor 1.2 use `declare_program!` or classic `declare_id!`? Confirm against installed docs before task 24 writes the scaffold</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>23 Freeze the Interface Contract</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Is the event emission API still `emit!(AccessLogged {...})` in 1.x?</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>24 Solana Program Scaffold</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Confirm whether Anchor 1.2 requires `declare_program!` with an IDL file, or classic `declare_id!`</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>24 Solana Program Scaffold</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Does `anchor build` need platform tools (`cargo-build-sbf`) installed separately?</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>24 Solana Program Scaffold</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Should the IDL be committed at scaffold time or after task 27?</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>25 Pure Hash Chain Module</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Should `chain_head` use SHA-256 directly or a domain-separated variant? Direct SHA-256 matches the contract and keeps client and program identical</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>25 Pure Hash Chain Module</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Should `verify_chain` live here or in a later task? Contract puts it here</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>26 Durable Outbox and Solana Flusher</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Flush on write plus a periodic sweep, or a fixed timer? The former gives snappy demo behavior without hammering devnet</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>26 Durable Outbox and Solana Flusher</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Retain pending events for how long before giving up?</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>26 Durable Outbox and Solana Flusher</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Batch multiple events per transaction to save fees, at the cost of per-event atomicity?</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>27 Build the Anchor Program</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Should `record_access` cap `event_count` or payload age?</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>27 Build the Anchor Program</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Emit the full `AccessEvent` on-chain, or only the hash with detail in Postgres?</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>28 Devnet Deploy</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Which devnet RPC provider for the app and E2E?</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>28 Devnet Deploy</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Record the exact deploy command in the README so the deployment is reproducible?</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>29 Solana Program Tests</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Coverage threshold for the Rust program? The TS side uses 70%; mirror it?</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>29 Solana Program Tests</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Should the tamper test live in Rust, TypeScript, or both? Both proves client and program agree</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>30 Solana Client and Environment</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Cache the head hash or read per request? Per request is simpler and current enough</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>30 Solana Client and Environment</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Should health fail loudly when the program is missing, or degrade to `status: degraded`?</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>31 Remove the Homemade Blockchain</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Keep the two-server demo or drop to one and reclaim the time? Recommendation: keep, it is the HA story</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>31 Remove the Homemade Blockchain</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Should `AccessLog` rows exist for pending events, or only anchored ones?</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>32 Wire Flusher to the Solana Program</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Flush immediately on write plus a periodic sweep, or on a fixed interval?</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>32 Wire Flusher to the Solana Program</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>What is acceptable pending lag before the demo looks wrong?</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>33 Patient Wallet Integration</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Does consent need revoking? Revocation on-chain is a real design problem, likely out of scope</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>33 Patient Wallet Integration</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Should patients read their own log entries directly from chain, bypassing the app?</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>34 Solana Verification UI</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Should the chain panel be visible to staff too, or patients only?</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>34 Solana Verification UI</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Poll for pending entries or rely on the socket? Socket is smoother if the flusher emits</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>35 E2E and Submission Disclosure</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Do the devnet specs need a funded CI wallet, or should the demo account be a documented devnet address?</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>35 E2E and Submission Disclosure</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Should the specs live in `e2e/solana/` as a separate directory?</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>36 Hackathon Documentation</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Remove the course logbooks from the fork; keep `gruppkontrakt.md` and the meeting notes for honest provenance</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>36 Hackathon Documentation</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Mermaid in markdown, or a rendered image? Mermaid renders on GitHub and stays current</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>37 Hackathon Submission and Decks</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Target the University award explicitly, or let it follow from the work?</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>37 Hackathon Submission and Decks</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Which track: Solana, or a general submission? Solana is a separate $100k pool</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>37 Hackathon Submission and Decks</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Is the repo public? It must be, or `hackathon@colosseum.com` needs access</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D77"/>
+  <autoFilter ref="A1:D112"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: translate to English and replace Graphify with Ripwire (task 36) (#3)
- Replace Graphify with Ripwire: delete graphify-out, commit
  ripwire-out/{graph.html,GRAPH_REPORT.md}, add npm run ripwire[:graph|:report],
  docs/ripwire.md, and a root AGENTS.md agent quick-start
- Rewrite docs/ARCHITECTURE_REVIEW.md around ripwire and update all references
- Translate API, database, raw-requirements, group-contract, meeting notes and
  remaining draft-task text to English; switch diacritic example to Polish
- Remove the course logbooks (docs/logbooks/) and fix dangling references
- Regenerate task-dependencies/task-gantt diagrams and the stakeholder report
- Correct stale demo captions (p2p/ledger) to the Solana topology
</commit_message>
<xml_diff>
--- a/docs/stakeholder-report.xlsx
+++ b/docs/stakeholder-report.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Changelog" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Tasks" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Questions" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Changelog" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Questions" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Tasks'!$A$1:$L$22</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Questions'!$A$1:$D$77</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Changelog'!$A$1:$E$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Tasks'!$A$1:$L$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Questions'!$A$1:$D$112</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -23,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -42,9 +43,6 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-    </font>
-    <font>
-      <i val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -72,12 +70,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -443,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -467,7 +464,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated 2026-09-03 08:13 UTC  |  matdevstamp/inl-3-awesome-journal</t>
+          <t>Generated 2026-10-11 17:09 UTC  |  matdevstamp/inl-3-awesome-journal</t>
         </is>
       </c>
     </row>
@@ -523,22 +520,22 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" t="n">
+        <v>19</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
         <v>4</v>
       </c>
-      <c r="D6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" t="n">
+      <c r="G6" t="n">
         <v>3</v>
-      </c>
-      <c r="F6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" t="n">
-        <v>20</v>
       </c>
     </row>
     <row r="7"/>
@@ -609,13 +606,13 @@
         <v>0</v>
       </c>
       <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
         <v>3</v>
       </c>
-      <c r="E10" t="n">
+      <c r="F10" t="n">
         <v>0</v>
-      </c>
-      <c r="F10" t="n">
-        <v>2</v>
       </c>
       <c r="G10" t="n">
         <v>0</v>
@@ -623,11 +620,7 @@
       <c r="H10" t="n">
         <v>2</v>
       </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>2026-09-04</t>
-        </is>
-      </c>
+      <c r="I10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -639,28 +632,24 @@
         <v>7</v>
       </c>
       <c r="C11" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="D11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E11" t="n">
+        <v>7</v>
+      </c>
+      <c r="F11" t="n">
         <v>0</v>
-      </c>
-      <c r="F11" t="n">
-        <v>1</v>
       </c>
       <c r="G11" t="n">
         <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>7</v>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>2026-09-05</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -672,13 +661,13 @@
         <v>6</v>
       </c>
       <c r="C12" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="D12" t="n">
         <v>0</v>
       </c>
       <c r="E12" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F12" t="n">
         <v>0</v>
@@ -687,13 +676,9 @@
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>6</v>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>2026-09-16</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -717,14 +702,14 @@
         <v>0</v>
       </c>
       <c r="G13" t="n">
+        <v>2</v>
+      </c>
+      <c r="H13" t="n">
         <v>0</v>
       </c>
-      <c r="H13" t="n">
-        <v>2</v>
-      </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -738,13 +723,13 @@
         <v>3</v>
       </c>
       <c r="C14" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D14" t="n">
         <v>0</v>
       </c>
       <c r="E14" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F14" t="n">
         <v>0</v>
@@ -753,111 +738,110 @@
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>3</v>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-    </row>
-    <row r="15"/>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+        <v>1</v>
+      </c>
+      <c r="I14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>16</v>
+      </c>
+      <c r="C15" t="n">
+        <v>16</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" t="n">
+        <v>2</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="16"/>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>Streams (ownership)</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>Stream</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>Tasks</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="C18" s="3" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr">
+      <c r="D18" s="3" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="E17" s="3" t="inlineStr">
+      <c r="E18" s="3" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
       </c>
-      <c r="F17" s="3" t="inlineStr">
+      <c r="F18" s="3" t="inlineStr">
         <is>
           <t>Blocked</t>
         </is>
       </c>
-      <c r="G17" s="3" t="inlineStr">
+      <c r="G18" s="3" t="inlineStr">
         <is>
           <t>Overdue</t>
         </is>
       </c>
-      <c r="H17" s="3" t="inlineStr">
+      <c r="H18" s="3" t="inlineStr">
         <is>
           <t>Next deadline</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>A-Identity</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>2</v>
-      </c>
-      <c r="C18" t="n">
-        <v>2</v>
-      </c>
-      <c r="D18" t="n">
-        <v>0</v>
-      </c>
-      <c r="E18" t="n">
-        <v>0</v>
-      </c>
-      <c r="F18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G18" t="n">
-        <v>0</v>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>2026-09-16</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>B-Patient</t>
+          <t>A-Identity</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D19" t="n">
         <v>0</v>
       </c>
       <c r="E19" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F19" t="n">
         <v>0</v>
@@ -865,29 +849,25 @@
       <c r="G19" t="n">
         <v>0</v>
       </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
+      <c r="H19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>C-Notes</t>
+          <t>B-Patient</t>
         </is>
       </c>
       <c r="B20" t="n">
         <v>1</v>
       </c>
       <c r="C20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D20" t="n">
         <v>0</v>
       </c>
       <c r="E20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F20" t="n">
         <v>0</v>
@@ -895,29 +875,25 @@
       <c r="G20" t="n">
         <v>0</v>
       </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
+      <c r="H20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>D-Audit</t>
+          <t>C-Notes</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C21" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D21" t="n">
         <v>0</v>
       </c>
       <c r="E21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F21" t="n">
         <v>0</v>
@@ -925,39 +901,61 @@
       <c r="G21" t="n">
         <v>0</v>
       </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>2026-09-16</t>
-        </is>
-      </c>
+      <c r="H21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>D-Audit</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="C22" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="D22" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F22" t="n">
         <v>0</v>
-      </c>
-      <c r="F22" t="n">
-        <v>3</v>
       </c>
       <c r="G22" t="n">
         <v>0</v>
       </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>2026-09-04</t>
+      <c r="H22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>31</v>
+      </c>
+      <c r="C23" t="n">
+        <v>18</v>
+      </c>
+      <c r="D23" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" t="n">
+        <v>13</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" t="n">
+        <v>4</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -972,14 +970,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -992,7 +990,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Compared against the snapshot of 2026-09-03 08:12 UTC</t>
+          <t>Compared against the snapshot of 2026-10-11 16:58 UTC</t>
         </is>
       </c>
     </row>
@@ -1025,13 +1023,145 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>No changes since the previous export.</t>
-        </is>
-      </c>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Questions</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>13 Patient View &amp; Search</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Question added</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>How to handle Polish characters in search? (ł, ż, ó)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Questions</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>13 Patient View &amp; Search</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Question removed</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>How to handle Swedish characters in search? (å, ä, ö)</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Questions</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>17 User Roles &amp; Access Control</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Question added</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>How to handle organization-based access for primary care centre? Answered: primary care centre is the login role</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Questions</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>17 User Roles &amp; Access Control</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Question removed</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>How to handle organization-based access for vårdcentral? Answered: vårdcentral is the login role</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Questions</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>36 Hackathon Documentation</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Question added</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Remove the course logbooks from the fork; keep `gruppkontrakt.md` and the meeting notes for honest provenance</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Questions</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>36 Hackathon Documentation</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Question removed</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Keep `gruppkontrakt.md` and the course logbooks in the fork, or remove them? Leaving them is honest; removing reduces noise</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:E10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1042,18 +1172,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L22"/>
+  <dimension ref="A1:L38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="39" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="37" customWidth="1" min="6" max="6"/>
+    <col width="47" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="48" customWidth="1" min="11" max="11"/>
     <col width="16" customWidth="1" min="12" max="12"/>
@@ -1140,7 +1270,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -1188,7 +1318,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -1235,22 +1365,22 @@
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Graphify Architecture Artifacts</t>
+          <t>Ripwire Architecture Artifacts</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Scaffold pair (Person 1 + Person 2)</t>
+          <t>Team (Gate 1 — Matias coordinates)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -1265,7 +1395,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>#30</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -1296,17 +1426,17 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>matdevstamp</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -1343,22 +1473,22 @@
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Vite + Tailwind CSS + shadcn/ui Setup</t>
+          <t>Next.js + Tailwind CSS + shadcn/ui Setup</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>matdevstamp</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -1372,7 +1502,11 @@
         </is>
       </c>
       <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>https://github.com/matdevstamp/inl-3-awesome-journal/issues/6</t>
+        </is>
+      </c>
       <c r="L6" t="n">
         <v>3</v>
       </c>
@@ -1391,22 +1525,22 @@
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Backend Project Setup</t>
+          <t>Backend Project Setup (Next.js Route Handlers &amp; Services)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>matdevstamp</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1416,11 +1550,15 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>#4, 05</t>
+          <t>#4, #6</t>
         </is>
       </c>
       <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>https://github.com/matdevstamp/inl-3-awesome-journal/issues/7</t>
+        </is>
+      </c>
       <c r="L7" t="n">
         <v>3</v>
       </c>
@@ -1444,17 +1582,17 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>matdevstamp</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1464,11 +1602,15 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>05, 06</t>
+          <t>#6, #7</t>
         </is>
       </c>
       <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>https://github.com/matdevstamp/inl-3-awesome-journal/issues/8</t>
+        </is>
+      </c>
       <c r="L8" t="n">
         <v>3</v>
       </c>
@@ -1492,12 +1634,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>matdevstamp</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1512,11 +1654,15 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>05, 07</t>
+          <t>#6, #8</t>
         </is>
       </c>
       <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>https://github.com/matdevstamp/inl-3-awesome-journal/issues/9</t>
+        </is>
+      </c>
       <c r="L9" t="n">
         <v>3</v>
       </c>
@@ -1540,17 +1686,17 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>matdevstamp</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1560,15 +1706,19 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>05, 06, 07, 08</t>
+          <t>#6, #7, #8, #9</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>10, 19</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr"/>
+          <t>#11, #29</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>https://github.com/matdevstamp/inl-3-awesome-journal/issues/10</t>
+        </is>
+      </c>
       <c r="L10" t="n">
         <v>4</v>
       </c>
@@ -1592,17 +1742,17 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>matdevstamp</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1612,15 +1762,19 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>05, 08, 07, 06</t>
+          <t>#6, #9, #8, #7</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>09</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr"/>
+          <t>#10</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>https://github.com/matdevstamp/inl-3-awesome-journal/issues/11</t>
+        </is>
+      </c>
       <c r="L11" t="n">
         <v>3</v>
       </c>
@@ -1648,17 +1802,17 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Kassim10</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1668,11 +1822,15 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>#4, 07, 06</t>
+          <t>#4, #8, #7</t>
         </is>
       </c>
       <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>https://github.com/matdevstamp/inl-3-awesome-journal/issues/13</t>
+        </is>
+      </c>
       <c r="L12" t="n">
         <v>4</v>
       </c>
@@ -1700,17 +1858,17 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>rcilomba</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1720,11 +1878,15 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>05, 07, 06</t>
+          <t>#6, #8, #7</t>
         </is>
       </c>
       <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>https://github.com/matdevstamp/inl-3-awesome-journal/issues/14</t>
+        </is>
+      </c>
       <c r="L13" t="n">
         <v>4</v>
       </c>
@@ -1752,17 +1914,17 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>rcilomba</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1772,15 +1934,19 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>#4, 11, 12</t>
+          <t>#4, #13, #14</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr"/>
+          <t>#16</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>https://github.com/matdevstamp/inl-3-awesome-journal/issues/15</t>
+        </is>
+      </c>
       <c r="L14" t="n">
         <v>4</v>
       </c>
@@ -1808,17 +1974,17 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Kassim10 (backend visibility) + rcilomba (UI)</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1828,15 +1994,19 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>#4, 11, 12</t>
+          <t>#4, #13, #14</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr"/>
+          <t>#15</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>https://github.com/matdevstamp/inl-3-awesome-journal/issues/16</t>
+        </is>
+      </c>
       <c r="L15" t="n">
         <v>4</v>
       </c>
@@ -1864,17 +2034,17 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>umoraghad0-del (huvudansvar, Stream D)</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1884,7 +2054,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>#4, 07, 06</t>
+          <t>#4, #8, #7</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -1892,7 +2062,11 @@
           <t>18</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr"/>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>https://github.com/matdevstamp/inl-3-awesome-journal/issues/17</t>
+        </is>
+      </c>
       <c r="L16" t="n">
         <v>4</v>
       </c>
@@ -1920,17 +2094,17 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>umoraghad0-del (pair-programmering)</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1940,11 +2114,15 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>15, 06</t>
+          <t>#17, #7</t>
         </is>
       </c>
       <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>https://github.com/matdevstamp/inl-3-awesome-journal/issues/18</t>
+        </is>
+      </c>
       <c r="L17" t="n">
         <v>4</v>
       </c>
@@ -1973,12 +2151,12 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>rcilomba</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1988,7 +2166,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>11, 12, 13, 14</t>
+          <t>#13, #14, #15, #16</t>
         </is>
       </c>
       <c r="J18" t="inlineStr"/>
@@ -2021,12 +2199,12 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>umoraghad0-del (pair-programmering)</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -2036,12 +2214,12 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>17, 14, 16, 12</t>
+          <t>#16, #18, #14, 17</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>#17</t>
         </is>
       </c>
       <c r="K19" t="inlineStr"/>
@@ -2068,17 +2246,17 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Team</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -2088,15 +2266,19 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>17, 15, 16, 18</t>
+          <t>#17, #18, 17, 18</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>09, 20</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr"/>
+          <t>#10, #30</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>https://github.com/matdevstamp/inl-3-awesome-journal/issues/29</t>
+        </is>
+      </c>
       <c r="L20" t="n">
         <v>4</v>
       </c>
@@ -2120,12 +2302,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Kassim10</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -2145,10 +2327,14 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>#3, 19</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr"/>
+          <t>#3, #29</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>https://github.com/matdevstamp/inl-3-awesome-journal/issues/30</t>
+        </is>
+      </c>
       <c r="L21" t="n">
         <v>4</v>
       </c>
@@ -2172,12 +2358,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Team</t>
+          <t>Kassim10</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -2192,17 +2378,845 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>19, 09, 20</t>
+          <t>#29, #10, #30</t>
         </is>
       </c>
       <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>https://github.com/matdevstamp/inl-3-awesome-journal/issues/31</t>
+        </is>
+      </c>
       <c r="L22" t="n">
         <v>4</v>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Solana Repo Split and Toolchain</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>matdevstamp</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>5h</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Freeze the Interface Contract</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>matdevstamp</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>3h</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>24, 25</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Solana Program Scaffold</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>matdevstamp</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>4h</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Pure Hash Chain Module</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>matdevstamp</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>5h</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Durable Outbox and Solana Flusher</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>matdevstamp</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>9h</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Build the Anchor Program</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>matdevstamp</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>5h</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>24, 25</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>28, 29</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Devnet Deploy</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>matdevstamp</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>2h</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Solana Program Tests</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>matdevstamp</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>7h</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>27, 28</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr"/>
+      <c r="L30" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Solana Client and Environment</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>matdevstamp</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>5h</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>27, 28</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Remove the Homemade Blockchain</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>matdevstamp</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>6h</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Wire Flusher to the Solana Program</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>matdevstamp</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>5h</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>31, 30</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr"/>
+      <c r="L33" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Patient Wallet Integration</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>matdevstamp</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>6h</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr"/>
+      <c r="L34" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr"/>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Solana Verification UI</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>matdevstamp</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>6h</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr"/>
+      <c r="L35" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>E2E and Submission Disclosure</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>matdevstamp</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>4h</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>29, 32</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>36, 37</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr"/>
+      <c r="L36" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr"/>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Hackathon Documentation</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>matdevstamp</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>5h</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>35, 37</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr"/>
+      <c r="L37" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr"/>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Hackathon Submission and Decks</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>matdevstamp</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>13h</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>35, 36</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr"/>
+      <c r="L38" t="n">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L22"/>
+  <autoFilter ref="A1:L38"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2213,11 +3227,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D77"/>
+  <dimension ref="A1:D112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="2" max="2"/>
     <col width="48" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
   </cols>
@@ -2257,12 +3271,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Which frontend framework will we use? (React, Vue, Svelte?)</t>
+          <t>Frontend: React inside Next.js (fullstack) — decided at kickoff</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2279,12 +3293,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Which authentication method? (JWT, sessions, passwordless?)</t>
+          <t>Auth: JWT in an httpOnly cookie — decided at kickoff</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2301,12 +3315,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>How will we handle the blockchain implementation?</t>
+          <t>Blockchain: simple custom chain (stream D split TBD) — decided at kickoff</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2323,12 +3337,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>What database will we use? (PostgreSQL, MySQL, SQLite?)</t>
+          <t>Database: PostgreSQL (dev + prod) — decided at kickoff</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2345,12 +3359,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Which database do we choose? (SQLite, PostgreSQL, or both?)</t>
+          <t>Which database do we choose? → **PostgreSQL** (dev and prod)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2372,7 +3386,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2394,7 +3408,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2416,7 +3430,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2428,17 +3442,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>03 Graphify Architecture Artifacts</t>
+          <t>03 Ripwire Architecture Artifacts</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Which graphify version and command will be documented in the README?</t>
+          <t>Which ripwire version and command will be documented in the README? Answer: `npm run ripwire` (ripwire 0.5.0), see `docs/ripwire.md`.</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2455,12 +3469,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>PostgreSQL vs SQLite? (see task 02-database-choice-discussion.md)</t>
+          <t>PostgreSQL vs SQLite? → **PostgreSQL** (see task 02-database-choice-discussion.md)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2477,12 +3491,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Should we use Prisma as the single source of truth?</t>
+          <t>Prisma as single source of truth? → yes; DBML dropped</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2504,7 +3518,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2526,7 +3540,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2538,7 +3552,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>05 Vite + Tailwind CSS + shadcn/ui Setup</t>
+          <t>05 Next.js + Tailwind CSS + shadcn/ui Setup</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2548,7 +3562,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2560,7 +3574,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>05 Vite + Tailwind CSS + shadcn/ui Setup</t>
+          <t>05 Next.js + Tailwind CSS + shadcn/ui Setup</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2570,7 +3584,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2582,7 +3596,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>05 Vite + Tailwind CSS + shadcn/ui Setup</t>
+          <t>05 Next.js + Tailwind CSS + shadcn/ui Setup</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2592,7 +3606,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2604,17 +3618,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>06 Backend Project Setup</t>
+          <t>06 Backend Project Setup (Next.js Route Handlers &amp; Services)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>PostgreSQL vs SQLite for development?</t>
+          <t>PostgreSQL vs SQLite for development? → PostgreSQL (task 02 decision)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2626,17 +3640,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>06 Backend Project Setup</t>
+          <t>06 Backend Project Setup (Next.js Route Handlers &amp; Services)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Which ORM to use? (Prisma recommended)</t>
+          <t>Which ORM to use? → Prisma</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2648,7 +3662,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>06 Backend Project Setup</t>
+          <t>06 Backend Project Setup (Next.js Route Handlers &amp; Services)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2658,7 +3672,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2680,7 +3694,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2702,7 +3716,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2724,7 +3738,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2746,7 +3760,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2768,7 +3782,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2790,7 +3804,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2812,7 +3826,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2834,7 +3848,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2856,7 +3870,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2878,7 +3892,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2900,7 +3914,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2917,12 +3931,12 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Which hosting platform for deployment?</t>
+          <t>Should we run E2E tests in CI from the start or only near Gate 4?</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2939,12 +3953,12 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Should we run E2E tests in CI?</t>
+          <t>Can the ruleset enforce the docs-direct carve-out per path?</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2961,12 +3975,12 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>JWT vs session-based auth? (JWT recommended for simplicity)</t>
+          <t>JWT vs session-based auth? → JWT in httpOnly cookie (kickoff)</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3027,12 +4041,12 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Should we use an API framework like Fastify instead of Express?</t>
+          <t>Express vs another framework? → no Express; Next.js route handlers (kickoff)</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3049,12 +4063,12 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>React vs Vue vs Svelte? (React recommended)</t>
+          <t>React vs Vue vs Svelte? → React in Next.js (kickoff)</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3071,12 +4085,12 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Which CSS framework? (Tailwind recommended)</t>
+          <t>Which CSS framework? → Tailwind + shadcn/ui (kickoff)</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3093,12 +4107,12 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>State management approach? (Context API vs Redux)</t>
+          <t>State management approach? → custom useSyncExternalStore session store; TanStack Query not adopted (PR #24)</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3115,12 +4129,12 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Should we use a component library? (Material UI, Ant Design?)</t>
+          <t>Component library? → shadcn/ui (kickoff)</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3137,7 +4151,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>How to handle Swedish characters in search? (å, ä, ö)</t>
+          <t>How to handle Polish characters in search? (ł, ż, ó)</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -3489,12 +4503,12 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>How to handle organization-based access for vårdcentral?</t>
+          <t>How to handle organization-based access for primary care centre? Answered: primary care centre is the login role</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3577,7 +4591,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Should we use Redis adapter for scaling?</t>
+          <t>Should we use Redis adapter for scaling? (open — single-pair demo works without it)</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -3599,12 +4613,12 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>How to handle socket authentication?</t>
+          <t>How to handle socket authentication? (JWT session cookie verified at handshake + peer shared secret for P2P calls)</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3621,12 +4635,12 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>What's the reconnection strategy?</t>
+          <t>What's the reconnection strategy? (socket.io-client auto-reconnect, 5 attempts, client-side note dedup on resync)</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3643,7 +4657,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Should we implement message acknowledgments?</t>
+          <t>Should we implement message acknowledgments? (open — current flow relies on client-side dedup instead)</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -3665,12 +4679,12 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Which testing framework to use? (Jest recommended for Node.js)</t>
+          <t>Which testing framework to use? → Vitest (unit/integration) + Playwright (E2E), matching task 09.</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3687,12 +4701,12 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>How to set up test database?</t>
+          <t>How to set up test database? → Docker Postgres via `e2e/global-setup.ts`, migrated and seeded per run.</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3709,12 +4723,12 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Should we implement E2E tests with Cypress?</t>
+          <t>Should we implement E2E tests with Cypress? → No, Playwright was already chosen in task 09.</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3731,12 +4745,12 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>How to handle socket.io testing?</t>
+          <t>How to handle socket.io testing? → Two `next start` instances (3001/3002) with real Socket.io ports; cross-server delivery is asserted over a WebSocket client.</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3775,12 +4789,12 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>How detailed should API documentation be?</t>
+          <t>How detailed should API documentation be? → route-handler table in README</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3797,12 +4811,12 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Should we use a documentation generator (e.g., Swagger)?</t>
+          <t>Should we use a documentation generator? → no (shared types; kickoff)</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3819,12 +4833,12 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>How to format meeting notes consistently?</t>
+          <t>How to format meeting notes consistently? → `YYYY-MM-DD-&lt;meeting-type&gt;.md`; use the structure in [`docs/MEETING_TEMPLATE.md`](../MEETING_TEMPLATE.md) and keep raw transcripts in `docs/meetings/archive/`.</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3916,8 +4930,778 @@
         </is>
       </c>
     </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>22 Solana Repo Split and Toolchain</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Does `anchor build` require platform tools (`cargo install --locked --git https://github.com/anza-xyz/platform-tools`)?</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>22 Solana Repo Split and Toolchain</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Which devnet RPC provider for E2E? The public endpoint rate-limits under parallel tests</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>23 Freeze the Interface Contract</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Does Anchor 1.2 use `declare_program!` or classic `declare_id!`? Confirm against installed docs before task 24 writes the scaffold</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>23 Freeze the Interface Contract</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Is the event emission API still `emit!(AccessLogged {...})` in 1.x?</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>24 Solana Program Scaffold</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Confirm whether Anchor 1.2 requires `declare_program!` with an IDL file, or classic `declare_id!`</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>24 Solana Program Scaffold</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Does `anchor build` need platform tools (`cargo-build-sbf`) installed separately?</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>24 Solana Program Scaffold</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Should the IDL be committed at scaffold time or after task 27?</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>25 Pure Hash Chain Module</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Should `chain_head` use SHA-256 directly or a domain-separated variant? Direct SHA-256 matches the contract and keeps client and program identical</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>25 Pure Hash Chain Module</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Should `verify_chain` live here or in a later task? Contract puts it here</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>26 Durable Outbox and Solana Flusher</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Flush on write plus a periodic sweep, or a fixed timer? The former gives snappy demo behavior without hammering devnet</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>26 Durable Outbox and Solana Flusher</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Retain pending events for how long before giving up?</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>26 Durable Outbox and Solana Flusher</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Batch multiple events per transaction to save fees, at the cost of per-event atomicity?</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>27 Build the Anchor Program</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Should `record_access` cap `event_count` or payload age?</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>27 Build the Anchor Program</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Emit the full `AccessEvent` on-chain, or only the hash with detail in Postgres?</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>28 Devnet Deploy</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Which devnet RPC provider for the app and E2E?</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>28 Devnet Deploy</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Record the exact deploy command in the README so the deployment is reproducible?</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>29 Solana Program Tests</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Coverage threshold for the Rust program? The TS side uses 70%; mirror it?</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>29 Solana Program Tests</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Should the tamper test live in Rust, TypeScript, or both? Both proves client and program agree</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>30 Solana Client and Environment</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Cache the head hash or read per request? Per request is simpler and current enough</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>30 Solana Client and Environment</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Should health fail loudly when the program is missing, or degrade to `status: degraded`?</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>31 Remove the Homemade Blockchain</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Keep the two-server demo or drop to one and reclaim the time? Recommendation: keep, it is the HA story</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>31 Remove the Homemade Blockchain</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Should `AccessLog` rows exist for pending events, or only anchored ones?</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>32 Wire Flusher to the Solana Program</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Flush immediately on write plus a periodic sweep, or on a fixed interval?</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>32 Wire Flusher to the Solana Program</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>What is acceptable pending lag before the demo looks wrong?</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>33 Patient Wallet Integration</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Does consent need revoking? Revocation on-chain is a real design problem, likely out of scope</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>33 Patient Wallet Integration</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Should patients read their own log entries directly from chain, bypassing the app?</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>34 Solana Verification UI</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Should the chain panel be visible to staff too, or patients only?</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>34 Solana Verification UI</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Poll for pending entries or rely on the socket? Socket is smoother if the flusher emits</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>35 E2E and Submission Disclosure</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Do the devnet specs need a funded CI wallet, or should the demo account be a documented devnet address?</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>35 E2E and Submission Disclosure</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Should the specs live in `e2e/solana/` as a separate directory?</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>36 Hackathon Documentation</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Remove the course logbooks from the fork; keep `gruppkontrakt.md` and the meeting notes for honest provenance</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>36 Hackathon Documentation</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Mermaid in markdown, or a rendered image? Mermaid renders on GitHub and stays current</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>37 Hackathon Submission and Decks</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Target the University award explicitly, or let it follow from the work?</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>37 Hackathon Submission and Decks</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Which track: Solana, or a general submission? Solana is a separate $100k pool</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>37 Hackathon Submission and Decks</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Is the repo public? It must be, or `hackathon@colosseum.com` needs access</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D77"/>
+  <autoFilter ref="A1:D112"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>